<commit_message>
added results for домашняя птица including 07/2025
</commit_message>
<xml_diff>
--- a/Models/Птицы/results/Птица - Лучшие модели.xlsx
+++ b/Models/Птицы/results/Птица - Лучшие модели.xlsx
@@ -462,13 +462,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>9.369999999999999</v>
+        <v>13.02</v>
       </c>
       <c r="C2" t="n">
-        <v>9.27</v>
+        <v>12.73</v>
       </c>
       <c r="D2" t="n">
-        <v>10.53</v>
+        <v>13</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -483,13 +483,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>384.26</v>
+        <v>277.84</v>
       </c>
       <c r="C3" t="n">
-        <v>356.69</v>
+        <v>285.19</v>
       </c>
       <c r="D3" t="n">
-        <v>208.73</v>
+        <v>143.7</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -504,13 +504,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6.56</v>
+        <v>8.81</v>
       </c>
       <c r="C4" t="n">
-        <v>9.93</v>
+        <v>10.08</v>
       </c>
       <c r="D4" t="n">
-        <v>13.17</v>
+        <v>10.26</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -526,7 +526,7 @@
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="n">
-        <v>3.505499728190417e+21</v>
+        <v>6.464043096337895e+18</v>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
@@ -542,17 +542,17 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>8.359999999999999</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="C6" t="n">
-        <v>8.74</v>
+        <v>7.01</v>
       </c>
       <c r="D6" t="n">
-        <v>8.529999999999999</v>
+        <v>12.15</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>SARIMA</t>
         </is>
       </c>
     </row>
@@ -563,13 +563,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>54.28</v>
+        <v>56.93</v>
       </c>
       <c r="C7" t="n">
-        <v>168.59</v>
+        <v>1801.25</v>
       </c>
       <c r="D7" t="n">
-        <v>99.98999999999999</v>
+        <v>99.95</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -585,7 +585,7 @@
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="n">
-        <v>3.241854430252585e+19</v>
+        <v>1.700944266158386e+20</v>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
@@ -601,17 +601,17 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>423.8</v>
+        <v>168.34</v>
       </c>
       <c r="C9" t="n">
-        <v>780.23</v>
+        <v>131.51</v>
       </c>
       <c r="D9" t="n">
-        <v>1075.22</v>
+        <v>673.22</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>SARIMA</t>
         </is>
       </c>
     </row>
@@ -622,13 +622,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>17.5</v>
+        <v>25.54</v>
       </c>
       <c r="C10" t="n">
-        <v>19.32</v>
+        <v>28.21</v>
       </c>
       <c r="D10" t="n">
-        <v>23.15</v>
+        <v>32.7</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -643,13 +643,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>16.21</v>
+        <v>20.69</v>
       </c>
       <c r="C11" t="n">
-        <v>13.88</v>
+        <v>14.34</v>
       </c>
       <c r="D11" t="n">
-        <v>27.94</v>
+        <v>29.95</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -664,13 +664,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>10.48</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="C12" t="n">
-        <v>14.62</v>
+        <v>14.98</v>
       </c>
       <c r="D12" t="n">
-        <v>11.82</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -685,17 +685,17 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>27.36</v>
+        <v>18.29</v>
       </c>
       <c r="C13" t="n">
-        <v>29.56</v>
+        <v>14.9</v>
       </c>
       <c r="D13" t="n">
-        <v>36.41</v>
+        <v>15.23</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>SARIMA</t>
         </is>
       </c>
     </row>
@@ -706,17 +706,17 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>98.45999999999999</v>
+        <v>207.49</v>
       </c>
       <c r="C14" t="n">
-        <v>74.51000000000001</v>
+        <v>328.85</v>
       </c>
       <c r="D14" t="n">
-        <v>170.89</v>
+        <v>210.69</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SARIMA</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
@@ -727,13 +727,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>42.42</v>
+        <v>49.15</v>
       </c>
       <c r="C15" t="n">
-        <v>370.55</v>
+        <v>263.68</v>
       </c>
       <c r="D15" t="n">
-        <v>18483.84</v>
+        <v>22915.51</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -748,13 +748,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>5.13</v>
+        <v>7.37</v>
       </c>
       <c r="C16" t="n">
-        <v>7.11</v>
+        <v>7.45</v>
       </c>
       <c r="D16" t="n">
-        <v>13.46</v>
+        <v>11.73</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -769,17 +769,17 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>181.16</v>
+        <v>121.22</v>
       </c>
       <c r="C17" t="n">
-        <v>175.35</v>
+        <v>613.87</v>
       </c>
       <c r="D17" t="n">
-        <v>288.27</v>
+        <v>275.58</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SARIMA</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="n">
-        <v>1.638749917683986e+23</v>
+        <v>3.073956394307394e+16</v>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
@@ -807,13 +807,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>45.92</v>
+        <v>38.39</v>
       </c>
       <c r="C19" t="n">
-        <v>52.35</v>
+        <v>40.5</v>
       </c>
       <c r="D19" t="n">
-        <v>91.48999999999999</v>
+        <v>60.6</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -828,17 +828,17 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>96.06999999999999</v>
+        <v>44.78</v>
       </c>
       <c r="C20" t="n">
-        <v>89.63</v>
+        <v>47.31</v>
       </c>
       <c r="D20" t="n">
-        <v>93.5</v>
+        <v>52.94</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SARIMA</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
@@ -849,17 +849,17 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>74.15000000000001</v>
+        <v>24.55</v>
       </c>
       <c r="C21" t="n">
-        <v>74.95</v>
+        <v>33.17</v>
       </c>
       <c r="D21" t="n">
-        <v>40.34</v>
+        <v>31.45</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Prophet</t>
+          <t>HW</t>
         </is>
       </c>
     </row>

</xml_diff>